<commit_message>
Funcionamiento completo de la aplicacion
</commit_message>
<xml_diff>
--- a/INFORME DE ACTIVIDADES - copia.xlsx
+++ b/INFORME DE ACTIVIDADES - copia.xlsx
@@ -265,22 +265,22 @@
     <xf numFmtId="15" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -925,113 +925,113 @@
   <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32" style="4" customWidth="1"/>
+    <col min="1" max="1" width="43.28515625" style="4" customWidth="1"/>
     <col min="2" max="2" width="11.140625" style="16" customWidth="1"/>
     <col min="3" max="3" width="12.140625" style="4" customWidth="1"/>
     <col min="4" max="4" width="15.42578125" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14.7109375" style="4" customWidth="1"/>
     <col min="6" max="6" width="15.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.85546875" style="4" customWidth="1"/>
-    <col min="8" max="8" width="10.5703125" style="4" customWidth="1"/>
-    <col min="9" max="9" width="56.140625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="19.28515625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="39.85546875" style="4" customWidth="1"/>
     <col min="10" max="10" width="0.140625" style="4" customWidth="1"/>
     <col min="11" max="11" width="26.42578125" style="4" customWidth="1"/>
     <col min="12" max="16384" width="11.42578125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="17"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="22" t="s">
+      <c r="B2" s="17"/>
+      <c r="C2" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
     </row>
     <row r="3" spans="1:10" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="18" t="s">
+      <c r="B3" s="17"/>
+      <c r="C3" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="18"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="18"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="18"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="22" t="s">
+      <c r="B4" s="17"/>
+      <c r="C4" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="21" t="s">
+      <c r="B5" s="17"/>
+      <c r="C5" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="21"/>
-      <c r="I5" s="21"/>
-      <c r="J5" s="21"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="22" t="s">
+      <c r="B6" s="17"/>
+      <c r="C6" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="22"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
     </row>
     <row r="7" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
@@ -1093,61 +1093,61 @@
       <c r="A10" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="20"/>
+      <c r="J10" s="20"/>
     </row>
     <row r="11" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
     </row>
     <row r="13" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="21"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
@@ -1487,13 +1487,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:J4"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:J2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:J3"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="B11:J11"/>
     <mergeCell ref="B12:J12"/>
@@ -1503,9 +1496,16 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:J6"/>
     <mergeCell ref="B9:J9"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:J3"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="74" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="73" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
   </tableParts>

</xml_diff>

<commit_message>
Actualizaciones de la aplicacion
</commit_message>
<xml_diff>
--- a/INFORME DE ACTIVIDADES - copia.xlsx
+++ b/INFORME DE ACTIVIDADES - copia.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apoyosistemas\Documents\Python - copia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Sistema2021\H\Sistemas\ACTIVIDADES\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>FECHA</t>
   </si>
@@ -86,28 +86,7 @@
     <t>Vo Bo:</t>
   </si>
   <si>
-    <t>CONTRATO DE PRESTACIÓN DE SERVICIOS DE APOYO A LA GESTION PARA LA ASISTENCIA TECNICAEN TODA LA INFRAESTRUCTURA TECNOLÓGICA DE LA ADMINISTRACIÓN MUNICIPAL DE LA CEJA DEL TAMBO</t>
-  </si>
-  <si>
-    <t>STEVEN ALEJANDRO RUIZ RENDON</t>
-  </si>
-  <si>
-    <t>1,036,964,737</t>
-  </si>
-  <si>
-    <t>MARIO ALFONSO HENAO LOPEZ</t>
-  </si>
-  <si>
     <t>Supervisor contrato</t>
-  </si>
-  <si>
-    <t>2026.10.05.06.035</t>
-  </si>
-  <si>
-    <t>Febrero 2026</t>
-  </si>
-  <si>
-    <t>8 de Enero de 2026 al 7 de Febrero de 2026</t>
   </si>
 </sst>
 </file>
@@ -265,22 +244,22 @@
     <xf numFmtId="15" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -940,98 +919,88 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
     </row>
     <row r="3" spans="1:10" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="17"/>
-      <c r="C4" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
+      <c r="B4" s="20"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="18" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
     </row>
     <row r="7" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
@@ -1077,9 +1046,7 @@
       <c r="A9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="23" t="s">
-        <v>25</v>
-      </c>
+      <c r="B9" s="23"/>
       <c r="C9" s="23"/>
       <c r="D9" s="23"/>
       <c r="E9" s="23"/>
@@ -1093,61 +1060,57 @@
       <c r="A10" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
-      <c r="J10" s="20"/>
-    </row>
-    <row r="11" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="19"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
     </row>
     <row r="13" spans="1:10" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="21"/>
+        <v>19</v>
+      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="19"/>
+      <c r="G13" s="19"/>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="13"/>
@@ -1487,6 +1450,13 @@
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="C4:J4"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="C2:J2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="C3:J3"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="B11:J11"/>
     <mergeCell ref="B12:J12"/>
@@ -1496,13 +1466,6 @@
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="C6:J6"/>
     <mergeCell ref="B9:J9"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:J4"/>
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:J2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:J3"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="73" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>